<commit_message>
Removed samples that were not part of this study from the Excel sheet provided by Kelsey
Co-authored-by: Cynthia SC <bioinformatic2019@gmail.com>
Co-authored-by: Daianna Gonzalez-Padilla <glezdaianna@gmail.com>
</commit_message>
<xml_diff>
--- a/raw-data/sample_info/Visium_HYP_HB_03_22_2023_HRD.xlsx
+++ b/raw-data/sample_info/Visium_HYP_HB_03_22_2023_HRD.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10409"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10311"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/Neural_Plasticity/Molecular_Profiling/Habenula/Human/Visium_experiment/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/leocollado/Dropbox/Mac/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DD136F5-C097-3446-948A-7C21846DCB79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8238864-46E4-3340-9CCC-CD56F89574C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="34080" yWindow="3900" windowWidth="28800" windowHeight="17500" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-43460" yWindow="5660" windowWidth="41340" windowHeight="18060" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="57">
   <si>
     <t>Sample #</t>
   </si>
@@ -137,18 +137,6 @@
     <t>HYP_1v_hrd</t>
   </si>
   <si>
-    <t>SI-TT-G9</t>
-  </si>
-  <si>
-    <t>CCGGAGGAAG</t>
-  </si>
-  <si>
-    <t>TGCGGATGTT</t>
-  </si>
-  <si>
-    <t>AACATCCGCA</t>
-  </si>
-  <si>
     <t>Agilent [cDNA] pg/ul</t>
   </si>
   <si>
@@ -219,42 +207,6 @@
   </si>
   <si>
     <t>AGGTAACACT</t>
-  </si>
-  <si>
-    <t>SI-TT-A2</t>
-  </si>
-  <si>
-    <t>GTGGATCAAA</t>
-  </si>
-  <si>
-    <t>GCCAACCCTG</t>
-  </si>
-  <si>
-    <t>CAGGGTTGGC</t>
-  </si>
-  <si>
-    <t>SI-TT-H12</t>
-  </si>
-  <si>
-    <t>TGATGATTCA</t>
-  </si>
-  <si>
-    <t>GTAGGAGTCG</t>
-  </si>
-  <si>
-    <t>CGACTCCTAC</t>
-  </si>
-  <si>
-    <t>SI-TT-G12</t>
-  </si>
-  <si>
-    <t>CTTGCATAAA</t>
-  </si>
-  <si>
-    <t>ATCAGGGCTT</t>
-  </si>
-  <si>
-    <t>AAGCCCTGAT</t>
   </si>
   <si>
     <t>Sample 3 (1v_HB)</t>
@@ -264,7 +216,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -304,24 +256,9 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <i/>
       <sz val="12"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="12"/>
-      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -341,7 +278,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -414,19 +351,8 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="8">
+  <cellStyleXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
@@ -434,9 +360,8 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -480,40 +405,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="6" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="6" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="5" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="7" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="6" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="4" fontId="5" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="8">
+  <cellStyles count="7">
     <cellStyle name="Followed Hyperlink" xfId="2" builtinId="9" hidden="1"/>
     <cellStyle name="Followed Hyperlink" xfId="4" builtinId="9" hidden="1"/>
     <cellStyle name="Followed Hyperlink" xfId="6" builtinId="9" hidden="1"/>
@@ -521,7 +427,6 @@
     <cellStyle name="Hyperlink" xfId="3" builtinId="8" hidden="1"/>
     <cellStyle name="Hyperlink" xfId="5" builtinId="8" hidden="1"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Percent" xfId="7" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
@@ -542,13 +447,13 @@
     <xdr:from>
       <xdr:col>10</xdr:col>
       <xdr:colOff>30726</xdr:colOff>
-      <xdr:row>12</xdr:row>
+      <xdr:row>8</xdr:row>
       <xdr:rowOff>61451</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
       <xdr:colOff>594033</xdr:colOff>
-      <xdr:row>24</xdr:row>
+      <xdr:row>20</xdr:row>
       <xdr:rowOff>69811</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -585,13 +490,13 @@
     <xdr:from>
       <xdr:col>7</xdr:col>
       <xdr:colOff>20485</xdr:colOff>
-      <xdr:row>12</xdr:row>
+      <xdr:row>8</xdr:row>
       <xdr:rowOff>49981</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
       <xdr:colOff>419920</xdr:colOff>
-      <xdr:row>24</xdr:row>
+      <xdr:row>20</xdr:row>
       <xdr:rowOff>70834</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -628,14 +533,14 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>1259758</xdr:colOff>
-      <xdr:row>11</xdr:row>
+      <xdr:row>7</xdr:row>
       <xdr:rowOff>202381</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
       <xdr:colOff>92178</xdr:colOff>
-      <xdr:row>24</xdr:row>
-      <xdr:rowOff>9530</xdr:rowOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>9531</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -671,13 +576,13 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>16795</xdr:colOff>
-      <xdr:row>12</xdr:row>
+      <xdr:row>8</xdr:row>
       <xdr:rowOff>6555</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
       <xdr:colOff>153630</xdr:colOff>
-      <xdr:row>23</xdr:row>
+      <xdr:row>19</xdr:row>
       <xdr:rowOff>184355</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -1694,7 +1599,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AB153"/>
+  <dimension ref="A1:AB149"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.1640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="18.1640625" style="9" customWidth="1"/>
@@ -1745,16 +1650,16 @@
         <v>10</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="I1" s="7" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="J1" s="7" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="K1" s="5" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="L1" s="7" t="s">
         <v>11</v>
@@ -1766,13 +1671,13 @@
         <v>17</v>
       </c>
       <c r="O1" s="5" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="P1" s="5" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="Q1" s="5" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="R1" s="12" t="s">
         <v>13</v>
@@ -1793,417 +1698,101 @@
         <v>19</v>
       </c>
     </row>
-    <row r="2" spans="1:28" s="21" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="15" t="s">
-        <v>31</v>
-      </c>
-      <c r="B2" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="C2" s="15" t="s">
-        <v>30</v>
-      </c>
-      <c r="D2" s="15" t="s">
-        <v>28</v>
-      </c>
-      <c r="E2" s="15" t="s">
-        <v>5</v>
-      </c>
-      <c r="F2" s="16">
-        <v>15.91</v>
-      </c>
-      <c r="G2" s="15">
+    <row r="2" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A2" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="F2" s="3">
+        <v>16.309999999999999</v>
+      </c>
+      <c r="G2" s="2">
         <v>16</v>
       </c>
-      <c r="H2" s="15">
-        <v>1950.02</v>
-      </c>
-      <c r="I2" s="16">
-        <v>9</v>
-      </c>
-      <c r="J2" s="16">
-        <f>H2*I2</f>
-        <v>17550.18</v>
-      </c>
-      <c r="K2" s="16">
-        <f>(H2*I2*40)/1000</f>
-        <v>702.0071999999999</v>
-      </c>
-      <c r="L2" s="16">
-        <f>0.25*K2</f>
-        <v>175.50179999999997</v>
-      </c>
-      <c r="M2" s="15">
-        <v>15</v>
-      </c>
-      <c r="N2" s="15">
-        <v>443</v>
-      </c>
-      <c r="O2" s="15">
-        <v>3119.47</v>
-      </c>
-      <c r="P2" s="16">
-        <v>5</v>
-      </c>
-      <c r="Q2" s="17">
-        <f>O2*P2</f>
-        <v>15597.349999999999</v>
-      </c>
-      <c r="R2" s="15" t="s">
-        <v>32</v>
-      </c>
-      <c r="S2" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="T2" s="15" t="s">
-        <v>34</v>
-      </c>
-      <c r="U2" s="18" t="s">
-        <v>35</v>
-      </c>
-      <c r="V2" s="19">
-        <v>85</v>
-      </c>
-      <c r="W2" s="15">
-        <f>((V2/100)*5000*60000)</f>
-        <v>255000000</v>
-      </c>
-      <c r="X2" s="20"/>
-      <c r="Y2" s="20"/>
-      <c r="AA2" s="22"/>
-      <c r="AB2" s="22"/>
-    </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A3" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C3" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="D3" s="2" t="s">
+      <c r="H2" s="2">
+        <v>3572.77</v>
+      </c>
+      <c r="I2" s="3">
+        <v>2</v>
+      </c>
+      <c r="J2" s="17">
+        <f t="shared" ref="J2" si="0">H2*I2</f>
+        <v>7145.54</v>
+      </c>
+      <c r="K2" s="17">
+        <f t="shared" ref="K2" si="1">(H2*I2*40)/1000</f>
+        <v>285.82159999999999</v>
+      </c>
+      <c r="L2" s="17">
+        <f t="shared" ref="L2" si="2">0.25*K2</f>
+        <v>71.455399999999997</v>
+      </c>
+      <c r="M2" s="2">
+        <v>16</v>
+      </c>
+      <c r="N2" s="8">
+        <v>447</v>
+      </c>
+      <c r="O2" s="2">
+        <v>3269.89</v>
+      </c>
+      <c r="P2" s="3">
+        <v>2</v>
+      </c>
+      <c r="Q2" s="19">
+        <f t="shared" ref="Q2" si="3">O2*P2</f>
+        <v>6539.78</v>
+      </c>
+      <c r="R2" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="S2" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="T2" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="U2" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="V2" s="8">
+        <v>80</v>
+      </c>
+      <c r="W2" s="18">
+        <f t="shared" ref="W2" si="4">((V2/100)*5000*60000)</f>
+        <v>240000000</v>
+      </c>
+      <c r="X2"/>
+      <c r="Y2"/>
+      <c r="AA2" s="10"/>
+      <c r="AB2" s="10"/>
+    </row>
+    <row r="8" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A8" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="H8" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="E3" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="F3" s="3">
-        <v>15.52</v>
-      </c>
-      <c r="G3" s="2">
-        <v>15</v>
-      </c>
-      <c r="H3" s="2">
-        <v>4993.5200000000004</v>
-      </c>
-      <c r="I3" s="3">
-        <v>1</v>
-      </c>
-      <c r="J3" s="23">
-        <f t="shared" ref="J3:J6" si="0">H3*I3</f>
-        <v>4993.5200000000004</v>
-      </c>
-      <c r="K3" s="23">
-        <f t="shared" ref="K3:K6" si="1">(H3*I3*40)/1000</f>
-        <v>199.74080000000001</v>
-      </c>
-      <c r="L3" s="23">
-        <f t="shared" ref="L3:L6" si="2">0.25*K3</f>
-        <v>49.935200000000002</v>
-      </c>
-      <c r="M3" s="2">
-        <v>17</v>
-      </c>
-      <c r="N3" s="8">
-        <v>452</v>
-      </c>
-      <c r="O3" s="2">
-        <v>10418.27</v>
-      </c>
-      <c r="P3" s="3">
-        <v>2</v>
-      </c>
-      <c r="Q3" s="26">
-        <f t="shared" ref="Q3:Q6" si="3">O3*P3</f>
-        <v>20836.54</v>
-      </c>
-      <c r="R3" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="S3" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="T3" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="U3" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="V3" s="8">
-        <v>100</v>
-      </c>
-      <c r="W3" s="25">
-        <f t="shared" ref="W3:W6" si="4">((V3/100)*5000*60000)</f>
-        <v>300000000</v>
-      </c>
-      <c r="X3"/>
-      <c r="Y3"/>
-      <c r="AA3" s="10"/>
-      <c r="AB3" s="10"/>
-    </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A4" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C4" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="F4" s="3">
-        <v>15.54</v>
-      </c>
-      <c r="G4" s="2">
-        <v>15</v>
-      </c>
-      <c r="H4" s="2">
-        <v>5351.97</v>
-      </c>
-      <c r="I4" s="3">
-        <v>2</v>
-      </c>
-      <c r="J4" s="23">
-        <f t="shared" si="0"/>
-        <v>10703.94</v>
-      </c>
-      <c r="K4" s="23">
-        <f t="shared" si="1"/>
-        <v>428.15760000000006</v>
-      </c>
-      <c r="L4" s="23">
-        <f t="shared" si="2"/>
-        <v>107.03940000000001</v>
-      </c>
-      <c r="M4" s="2">
-        <v>16</v>
-      </c>
-      <c r="N4" s="8">
-        <v>429</v>
-      </c>
-      <c r="O4" s="2">
-        <v>9036.14</v>
-      </c>
-      <c r="P4" s="3">
-        <v>2</v>
-      </c>
-      <c r="Q4" s="26">
-        <f t="shared" si="3"/>
-        <v>18072.28</v>
-      </c>
-      <c r="R4" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="S4" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="T4" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="U4" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="V4" s="8">
-        <v>90</v>
-      </c>
-      <c r="W4" s="25">
-        <f t="shared" si="4"/>
-        <v>270000000</v>
-      </c>
-      <c r="X4"/>
-      <c r="Y4"/>
-      <c r="AA4" s="10"/>
-      <c r="AB4" s="10"/>
-    </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A5" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="C5" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="F5" s="3">
-        <v>16.309999999999999</v>
-      </c>
-      <c r="G5" s="2">
-        <v>16</v>
-      </c>
-      <c r="H5" s="2">
-        <v>3572.77</v>
-      </c>
-      <c r="I5" s="3">
-        <v>2</v>
-      </c>
-      <c r="J5" s="23">
-        <f t="shared" si="0"/>
-        <v>7145.54</v>
-      </c>
-      <c r="K5" s="23">
-        <f t="shared" si="1"/>
-        <v>285.82159999999999</v>
-      </c>
-      <c r="L5" s="23">
-        <f t="shared" si="2"/>
-        <v>71.455399999999997</v>
-      </c>
-      <c r="M5" s="2">
-        <v>16</v>
-      </c>
-      <c r="N5" s="8">
-        <v>447</v>
-      </c>
-      <c r="O5" s="2">
-        <v>3269.89</v>
-      </c>
-      <c r="P5" s="3">
-        <v>2</v>
-      </c>
-      <c r="Q5" s="26">
-        <f t="shared" si="3"/>
-        <v>6539.78</v>
-      </c>
-      <c r="R5" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="S5" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="T5" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="U5" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="V5" s="8">
-        <v>80</v>
-      </c>
-      <c r="W5" s="25">
-        <f t="shared" si="4"/>
-        <v>240000000</v>
-      </c>
-      <c r="X5"/>
-      <c r="Y5"/>
-      <c r="AA5" s="10"/>
-      <c r="AB5" s="10"/>
-    </row>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A6" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C6" s="6" t="s">
+      <c r="K8" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="D6" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="F6" s="2">
-        <v>15.24</v>
-      </c>
-      <c r="G6" s="2">
-        <v>15</v>
-      </c>
-      <c r="H6" s="2">
-        <v>3312.65</v>
-      </c>
-      <c r="I6" s="3">
-        <v>2</v>
-      </c>
-      <c r="J6" s="23">
-        <f t="shared" si="0"/>
-        <v>6625.3</v>
-      </c>
-      <c r="K6" s="23">
-        <f t="shared" si="1"/>
-        <v>265.012</v>
-      </c>
-      <c r="L6" s="23">
-        <f t="shared" si="2"/>
-        <v>66.253</v>
-      </c>
-      <c r="M6" s="2">
-        <v>17</v>
-      </c>
-      <c r="N6" s="2">
-        <v>429</v>
-      </c>
-      <c r="O6" s="2">
-        <v>7864.15</v>
-      </c>
-      <c r="P6" s="24">
-        <v>2</v>
-      </c>
-      <c r="Q6" s="26">
-        <f t="shared" si="3"/>
-        <v>15728.3</v>
-      </c>
-      <c r="R6" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="S6" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="T6" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="U6" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="V6" s="8">
-        <v>85</v>
-      </c>
-      <c r="W6" s="25">
-        <f t="shared" si="4"/>
-        <v>255000000</v>
-      </c>
-    </row>
-    <row r="12" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A12" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="D12" s="6" t="s">
-        <v>49</v>
-      </c>
-      <c r="H12" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="K12" s="2" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="153" ht="17" customHeight="1" x14ac:dyDescent="0.2"/>
+    </row>
+    <row r="149" ht="17" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -2245,7 +1834,7 @@
         <v>5</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="C2" s="3">
         <v>15.52</v>
@@ -2259,7 +1848,7 @@
         <v>6</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="C3" s="3">
         <v>15.54</v>
@@ -2273,7 +1862,7 @@
         <v>7</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="C4" s="3">
         <v>16.309999999999999</v>
@@ -2287,7 +1876,7 @@
         <v>8</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="C5" s="2">
         <v>15.24</v>
@@ -2352,16 +1941,16 @@
         <v>10</v>
       </c>
       <c r="U3" s="5" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="V3" s="7" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="W3" s="7" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="X3" s="5" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
     </row>
     <row r="4" spans="14:24" x14ac:dyDescent="0.2">
@@ -2403,16 +1992,16 @@
     </row>
     <row r="5" spans="14:24" x14ac:dyDescent="0.2">
       <c r="N5" s="2" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="O5" s="2" t="s">
         <v>29</v>
       </c>
       <c r="P5" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q5" s="2" t="s">
         <v>43</v>
-      </c>
-      <c r="Q5" s="2" t="s">
-        <v>47</v>
       </c>
       <c r="R5" s="2" t="s">
         <v>5</v>
@@ -2429,27 +2018,27 @@
       <c r="V5" s="3">
         <v>1</v>
       </c>
-      <c r="W5" s="23">
+      <c r="W5" s="17">
         <f t="shared" ref="W5:W8" si="0">U5*V5</f>
         <v>4993.5200000000004</v>
       </c>
-      <c r="X5" s="23">
+      <c r="X5" s="17">
         <f t="shared" ref="X5:X8" si="1">(U5*V5*40)/1000</f>
         <v>199.74080000000001</v>
       </c>
     </row>
     <row r="6" spans="14:24" x14ac:dyDescent="0.2">
       <c r="N6" s="2" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="O6" s="2" t="s">
         <v>29</v>
       </c>
       <c r="P6" s="6" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="Q6" s="2" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="R6" s="2" t="s">
         <v>6</v>
@@ -2466,27 +2055,27 @@
       <c r="V6" s="3">
         <v>2</v>
       </c>
-      <c r="W6" s="23">
+      <c r="W6" s="17">
         <f t="shared" si="0"/>
         <v>10703.94</v>
       </c>
-      <c r="X6" s="23">
+      <c r="X6" s="17">
         <f t="shared" si="1"/>
         <v>428.15760000000006</v>
       </c>
     </row>
     <row r="7" spans="14:24" x14ac:dyDescent="0.2">
       <c r="N7" s="2" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="O7" s="2" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="P7" s="6" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="Q7" s="2" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="R7" s="2" t="s">
         <v>7</v>
@@ -2503,27 +2092,27 @@
       <c r="V7" s="3">
         <v>2</v>
       </c>
-      <c r="W7" s="23">
+      <c r="W7" s="17">
         <f t="shared" si="0"/>
         <v>7145.54</v>
       </c>
-      <c r="X7" s="23">
+      <c r="X7" s="17">
         <f t="shared" si="1"/>
         <v>285.82159999999999</v>
       </c>
     </row>
     <row r="8" spans="14:24" x14ac:dyDescent="0.2">
       <c r="N8" s="2" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="O8" s="2" t="s">
         <v>29</v>
       </c>
       <c r="P8" s="6" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="Q8" s="2" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="R8" s="2" t="s">
         <v>8</v>
@@ -2540,11 +2129,11 @@
       <c r="V8" s="3">
         <v>2</v>
       </c>
-      <c r="W8" s="23">
+      <c r="W8" s="17">
         <f t="shared" si="0"/>
         <v>6625.3</v>
       </c>
-      <c r="X8" s="23">
+      <c r="X8" s="17">
         <f t="shared" si="1"/>
         <v>265.012</v>
       </c>
@@ -2585,39 +2174,39 @@
   <sheetData>
     <row r="5" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B5" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C5" t="s">
         <v>48</v>
-      </c>
-      <c r="C5" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="6" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B6" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C6" t="s">
         <v>49</v>
-      </c>
-      <c r="C6" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="7" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B7" s="2" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="C7" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
     </row>
     <row r="8" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B8" s="2" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="C8" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
     </row>
     <row r="36" spans="20:20" x14ac:dyDescent="0.2">
       <c r="T36" t="s">
-        <v>72</v>
+        <v>56</v>
       </c>
     </row>
   </sheetData>

</xml_diff>